<commit_message>
Correct helm and motorcycle spare parts admin rate to 8.25% and unit to 2.50% based on official table
</commit_message>
<xml_diff>
--- a/shopee_admin_fees_2026.xlsx
+++ b/shopee_admin_fees_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,17 +456,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Otomotif</t>
+          <t>Sepeda Motor</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Suku Cadang &amp; Aksesoris Motor/Mobil</t>
+          <t>Helm &amp; Suku Cadang Motor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Helm, Ban, Oli, Aksesoris Motor/Mobil</t>
+          <t>Helm, Aksesoris Pengendara, Busi, Aki, Ban Motor, Knalpot, Oli Motor, Rantai</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -476,54 +476,54 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>8.25%</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>9.25%</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>9.95%</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Tarif admin dasar kategori otomotif umum</t>
+          <t>Helm &amp; Suku Cadang Motor</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Elektronik (Audio)</t>
+          <t>Sepeda Motor</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Perangkat Audio &amp; Speaker</t>
+          <t>Sepeda Motor (Unit)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Speaker, Home Theater, Karaoke, AV Receiver</t>
+          <t>Unit Kendaraan Sepeda Motor</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Grup B</t>
+          <t>Grup Khusus</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Speaker dan perangkat audio utama</t>
+          <t>Unit kendaraan sepeda motor</t>
         </is>
       </c>
     </row>
@@ -535,12 +535,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mikrofon &amp; Aksesoris</t>
+          <t>Perangkat Audio &amp; Speaker</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mikrofon, Stand, Kabel Audio &amp; Mixer</t>
+          <t>Speaker, Home Theater, Karaoke, AV Receiver</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aksesoris perekaman dan alat audio</t>
+          <t>Speaker dan perangkat audio utama</t>
         </is>
       </c>
     </row>
@@ -572,32 +572,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Earphone &amp; Headphone</t>
+          <t>Mikrofon &amp; Aksesoris</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Earphone, Headphone, Headset, Handsfree</t>
+          <t>Mikrofon, Stand, Kabel Audio &amp; Mixer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Grup C</t>
+          <t>Grup B</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.75%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7.70%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Tarif lebih rendah untuk earphone/headphone</t>
+          <t>Aksesoris perekaman dan alat audio</t>
         </is>
       </c>
     </row>
@@ -609,106 +609,106 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Media Player</t>
+          <t>Earphone &amp; Headphone</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MP3 &amp; MP4 Player, CD/DVD/Blu-ray Player, Radio, Voice Recorder</t>
+          <t>Earphone, Headphone, Headset, Handsfree</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Grup B</t>
+          <t>Grup C</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>9.50%</t>
+          <t>6.75%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>7.70%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Tarif media player sedikit lebih tinggi</t>
+          <t>Tarif lebih rendah untuk earphone/headphone</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Elektronik (Kelistrikan)</t>
+          <t>Elektronik (Audio)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kelistrikan</t>
+          <t>Media Player</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Stop Kontak, Sambungan Kabel, Saklar, Alarm, Anti Petir</t>
+          <t>MP3 &amp; MP4 Player, CD/DVD/Blu-ray Player, Radio, Voice Recorder</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Grup A</t>
+          <t>Grup B</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>9.50%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Peralatan instalasi kelistrikan</t>
+          <t>Tarif media player sedikit lebih tinggi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aksesoris Fashion</t>
+          <t>Elektronik (Kelistrikan)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Aksesoris Rambut &amp; Perhiasan</t>
+          <t>Kelistrikan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Topi, Kacamata, Anting, Kalung, Gelang, Jepitan, Bros</t>
+          <t>Stop Kontak, Sambungan Kabel, Saklar, Alarm, Anti Petir</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Grup B</t>
+          <t>Grup A</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Aksesoris fashion umum non-logam mulia</t>
+          <t>Peralatan instalasi kelistrikan</t>
         </is>
       </c>
     </row>
@@ -720,12 +720,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Aksesoris Tambahan</t>
+          <t>Aksesoris Rambut &amp; Perhiasan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Masker Kain, Masker Medis</t>
+          <t>Topi, Kacamata, Anting, Kalung, Gelang, Jepitan, Bros</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -735,17 +735,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.25%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Tarif khusus untuk produk masker</t>
+          <t>Aksesoris fashion umum non-logam mulia</t>
         </is>
       </c>
     </row>
@@ -757,69 +757,69 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Logam Mulia</t>
+          <t>Aksesoris Tambahan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Emas Batangan, Berlian, Perak, Platinum, Perhiasan Berharga</t>
+          <t>Masker Kain, Masker Medis</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Grup E</t>
+          <t>Grup B</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>9.25%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Tarif admin sangat rendah untuk investasi mulia</t>
+          <t>Tarif khusus untuk produk masker</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Fashion Bayi &amp; Anak</t>
+          <t>Aksesoris Fashion</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pakaian &amp; Sepatu Anak</t>
+          <t>Logam Mulia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Baju Bayi, Pakaian Anak, Sepatu Anak, Sandal Anak, Kaos Kaki Anak</t>
+          <t>Emas Batangan, Berlian, Perak, Platinum, Perhiasan Berharga</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Grup B</t>
+          <t>Grup E</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Fashion khusus anak &amp; bayi</t>
+          <t>Tarif admin sangat rendah untuk investasi mulia</t>
         </is>
       </c>
     </row>
@@ -831,69 +831,69 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Aksesoris Perhiasan Anak</t>
+          <t>Pakaian &amp; Sepatu Anak</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Gelang Emas/Perak Anak, Anting Anak, Kalung Anak</t>
+          <t>Baju Bayi, Pakaian Anak, Sepatu Anak, Sandal Anak, Kaos Kaki Anak</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Grup E</t>
+          <t>Grup B</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Perhiasan berharga untuk anak/bayi</t>
+          <t>Fashion khusus anak &amp; bayi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fashion Muslim</t>
+          <t>Fashion Bayi &amp; Anak</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pakaian Muslim Dewasa &amp; Anak</t>
+          <t>Aksesoris Perhiasan Anak</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hijab, Gamis, Mukena, Perlengkapan Sholat, Koko, Sarung</t>
+          <t>Gelang Emas/Perak Anak, Anting Anak, Kalung Anak</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Grup B</t>
+          <t>Grup E</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>9.25%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Fashion muslim secara umum</t>
+          <t>Perhiasan berharga untuk anak/bayi</t>
         </is>
       </c>
     </row>
@@ -905,86 +905,86 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pakaian Olahraga Muslim</t>
+          <t>Pakaian Muslim Dewasa &amp; Anak</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Baju Olahraga Muslim Wanita, Baju Renang Muslim</t>
+          <t>Hijab, Gamis, Mukena, Perlengkapan Sholat, Koko, Sarung</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Grup A</t>
+          <t>Grup B</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>9.25%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Baju olahraga / renang muslim khusus</t>
+          <t>Fashion muslim secara umum</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jam Tangan</t>
+          <t>Fashion Muslim</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jam Tangan &amp; Aksesoris</t>
+          <t>Pakaian Olahraga Muslim</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Jam Tangan Pria, Wanita, Couple, Strap Jam, Baterai Jam</t>
+          <t>Baju Olahraga Muslim Wanita, Baju Renang Muslim</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Grup B</t>
+          <t>Grup A</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Seluruh jam tangan dan sparepartnya</t>
+          <t>Baju olahraga / renang muslim khusus</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Koper &amp; Tas Travel</t>
+          <t>Jam Tangan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Koper &amp; Aksesoris Travel</t>
+          <t>Jam Tangan &amp; Aksesoris</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Koper, Bantal Leher Travel, Tag Koper, Organizer, Pelindung Koper</t>
+          <t>Jam Tangan Pria, Wanita, Couple, Strap Jam, Baterai Jam</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Perlengkapan bagasi dan travel</t>
+          <t>Seluruh jam tangan dan sparepartnya</t>
         </is>
       </c>
     </row>
@@ -1016,69 +1016,69 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tas Duffel</t>
+          <t>Koper &amp; Aksesoris Travel</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tas Duffel Travel</t>
+          <t>Koper, Bantal Leher Travel, Tag Koper, Organizer, Pelindung Koper</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Grup A</t>
+          <t>Grup B</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Tas duffel besar</t>
+          <t>Perlengkapan bagasi dan travel</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Pakaian Pria &amp; Wanita</t>
+          <t>Koper &amp; Tas Travel</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pakaian Pria &amp; Wanita Dewasa</t>
+          <t>Tas Duffel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Kaos, Kemeja, Celana, Jaket, Blazer, Dress, Rok, Pakaian Dalam, Piyama</t>
+          <t>Tas Duffel Travel</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Grup B</t>
+          <t>Grup A</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>9.25%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Tarif admin pakaian dewasa utama</t>
+          <t>Tas duffel besar</t>
         </is>
       </c>
     </row>
@@ -1090,32 +1090,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kaos Kaki</t>
+          <t>Pakaian Pria &amp; Wanita Dewasa</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Kaos Kaki Pria/Wanita Dewasa</t>
+          <t>Kaos, Kemeja, Celana, Jaket, Blazer, Dress, Rok, Pakaian Dalam, Piyama</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Grup A</t>
+          <t>Grup B</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>9.25%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Tarif khusus kaos kaki</t>
+          <t>Tarif admin pakaian dewasa utama</t>
         </is>
       </c>
     </row>
@@ -1127,49 +1127,49 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Stocking</t>
+          <t>Kaos Kaki</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Stocking Wanita</t>
+          <t>Kaos Kaki Pria/Wanita Dewasa</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Grup B</t>
+          <t>Grup A</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Stocking wanita dewasa</t>
+          <t>Tarif khusus kaos kaki</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sepatu Pria &amp; Wanita</t>
+          <t>Pakaian Pria &amp; Wanita</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alas Kaki Dewasa</t>
+          <t>Stocking</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sepatu, Sandal, Sneakers, Boots, Loafer, Heels, Wedges, Flat Shoes</t>
+          <t>Stocking Wanita</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1189,24 +1189,24 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Sandal, sepatu dan aksesoris perawatan sepatu</t>
+          <t>Stocking wanita dewasa</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Tas Pria &amp; Wanita</t>
+          <t>Sepatu Pria &amp; Wanita</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tas &amp; Aksesoris Tas Dewasa</t>
+          <t>Alas Kaki Dewasa</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ransel, Clutch, Dompet, Tote Bag, Tas Selempang, Tas Laptop</t>
+          <t>Sepatu, Sandal, Sneakers, Boots, Loafer, Heels, Wedges, Flat Shoes</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1226,81 +1226,81 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Tas kerja, ransel, clutch dan dompet dewasa</t>
+          <t>Sandal, sepatu dan aksesoris perawatan sepatu</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Handphone &amp; Aksesoris</t>
+          <t>Tas Pria &amp; Wanita</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gadget &amp; Aksesoris</t>
+          <t>Tas &amp; Aksesoris Tas Dewasa</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Smartphone, Tablet, Casing, Charger, Kabel Data, Powerbank</t>
+          <t>Ransel, Clutch, Dompet, Tote Bag, Tas Selempang, Tas Laptop</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Grup D</t>
+          <t>Grup B</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>5.25%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>5.70%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Tarif elektronik gadget</t>
+          <t>Tas kerja, ransel, clutch dan dompet dewasa</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Makanan &amp; Minuman</t>
+          <t>Handphone &amp; Aksesoris</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kuliner &amp; FMCG</t>
+          <t>Gadget &amp; Aksesoris</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Snack, Camilan, Kopi, Teh, Sambal, Mie Instan</t>
+          <t>Smartphone, Tablet, Casing, Charger, Kabel Data, Powerbank</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Grup A</t>
+          <t>Grup D</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>5.25%</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>5.70%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Makanan minuman instan</t>
+          <t>Tarif elektronik gadget</t>
         </is>
       </c>
     </row>
@@ -1312,30 +1312,67 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>Kuliner &amp; FMCG</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Snack, Camilan, Kopi, Teh, Sambal, Mie Instan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Grup A</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>11.00%</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Makanan minuman instan</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Makanan &amp; Minuman</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>Sembako Pokok</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Beras, Minyak Goreng, Gula Pasir, Tepung</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Grup E</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>4.25%</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>4.20%</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Sembako bahan pokok</t>
         </is>

</xml_diff>